<commit_message>
Fix quotation printing and company week numbering
</commit_message>
<xml_diff>
--- a/public/quotation-template.xlsx
+++ b/public/quotation-template.xlsx
@@ -2,9 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotation" sheetId="1" r:id="R7193774b5ae649c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotation" sheetId="1" r:id="R980d05a300de405e"/>
   </x:sheets>
 </x:workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -21,7 +25,7 @@
     <x:numFmt numFmtId="181" formatCode="m/d/yy;@"/>
     <x:numFmt numFmtId="182" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </x:numFmts>
-  <x:fonts count="45">
+  <x:fonts count="48">
     <x:font>
       <x:sz val="10"/>
       <x:name val="Arial"/>
@@ -259,6 +263,22 @@
       <x:sz val="11"/>
       <x:color theme="1"/>
       <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="8"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Arial"/>
     </x:font>
   </x:fonts>
   <x:fills count="35">
@@ -735,7 +755,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="144">
+  <x:cellXfs count="159">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -1147,6 +1167,49 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="179" fontId="45" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="179" fontId="45" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="45" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="179" fontId="45" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="49">
@@ -1271,7 +1334,7 @@
 </x:styleSheet>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1288,13 +1351,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="/xl/media/image1.png"/>
+        <xdr:cNvPr id="1" name="/xl/media/image3.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Refc6c374fde94d83"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R83f9b71955dd4fc2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1320,13 +1383,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="/xl/media/image2.png"/>
+        <xdr:cNvPr id="2" name="/xl/media/image4.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R6c2f06bfa6574aa4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0a6c93e69c4c4bc5"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1552,7 +1615,7 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultColWidth="9.160714149475098" defaultRowHeight="16"/>
   <x:cols>
@@ -1579,11 +1642,21 @@
         </x:is>
       </x:c>
     </x:row>
-    <x:row r="3" s="1" customFormat="1" customHeight="1"/>
+    <x:row r="3" s="1" customFormat="1" customHeight="1">
+      <x:c r="B3" s="155" t="str">
+        <x:v>LORIOT INDUSTRIAL CO., LTD</x:v>
+      </x:c>
+      <x:c r="C3" s="155"/>
+      <x:c r="D3" s="155"/>
+      <x:c r="E3" s="155"/>
+    </x:row>
     <x:row r="4" s="2" customFormat="1" customHeight="1">
-      <x:c r="B4" s="13"/>
-      <x:c r="C4" s="13"/>
-      <x:c r="D4" s="14"/>
+      <x:c r="B4" s="158" t="str">
+        <x:v>129 TAN CANG STR, THANH MY TAY WARD, HCMC</x:v>
+      </x:c>
+      <x:c r="C4" s="158"/>
+      <x:c r="D4" s="155"/>
+      <x:c r="E4" s="155"/>
       <x:c r="F4" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">QUOTATION NO.</x:t>
@@ -1594,10 +1667,12 @@
       </x:c>
     </x:row>
     <x:row r="5" s="2" customFormat="1" customHeight="1">
-      <x:c r="B5" s="17"/>
-      <x:c r="C5" s="17"/>
-      <x:c r="D5" s="14"/>
-      <x:c r="E5" s="18"/>
+      <x:c r="B5" s="156" t="str">
+        <x:v>TEL: +84-28-3899 1163          FAX: +84-28-3899 1189</x:v>
+      </x:c>
+      <x:c r="C5" s="156"/>
+      <x:c r="D5" s="155"/>
+      <x:c r="E5" s="157"/>
       <x:c r="F5" s="14" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">DATE</x:t>
@@ -2087,7 +2162,6 @@
     <x:row r="98" s="3" customFormat="1" customHeight="1"/>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="B4:C4"/>
     <x:mergeCell ref="A14:B14"/>
     <x:mergeCell ref="E14:F14"/>
     <x:mergeCell ref="A15:B15"/>
@@ -2099,8 +2173,11 @@
     <x:mergeCell ref="A20:G20"/>
     <x:mergeCell ref="A36:H36"/>
     <x:mergeCell ref="B37:E37"/>
+    <x:mergeCell ref="B3:E3"/>
+    <x:mergeCell ref="B4:E4"/>
+    <x:mergeCell ref="B5:E5"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49309c9a63b543e0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fb6cb734d3d4df5"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fix quotation number label in Excel export
</commit_message>
<xml_diff>
--- a/public/quotation-template.xlsx
+++ b/public/quotation-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotation" sheetId="1" r:id="R980d05a300de405e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotation" sheetId="1" r:id="R0fd40f4dea194b41"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="181" formatCode="m/d/yy;@"/>
     <x:numFmt numFmtId="182" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </x:numFmts>
-  <x:fonts count="48">
+  <x:fonts count="50">
     <x:font>
       <x:sz val="10"/>
       <x:name val="Arial"/>
@@ -278,6 +278,16 @@
     <x:font>
       <x:sz val="8"/>
       <x:color rgb="FF111111"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FFA6A6A6"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="8"/>
+      <x:color rgb="FFA6A6A6"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -755,7 +765,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="159">
+  <x:cellXfs count="166">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -1210,6 +1220,27 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="46" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="48" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="49">
@@ -1351,13 +1382,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="/xl/media/image3.png"/>
+        <xdr:cNvPr id="1" name="/xl/media/image.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R83f9b71955dd4fc2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re34641f6b8fe4e78"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1383,13 +1414,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="/xl/media/image4.png"/>
+        <xdr:cNvPr id="2" name="/xl/media/image2.png"/>
         <xdr:cNvPicPr>
           <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0a6c93e69c4c4bc5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R27132b28be62416e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1656,12 +1687,10 @@
       </x:c>
       <x:c r="C4" s="158"/>
       <x:c r="D4" s="155"/>
-      <x:c r="E4" s="155"/>
-      <x:c r="F4" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">QUOTATION NO.</x:t>
-        </x:is>
-      </x:c>
+      <x:c r="E4" s="164" t="str">
+        <x:v>QUOTATION NO.</x:v>
+      </x:c>
+      <x:c r="F4" s="162"/>
       <x:c r="G4" s="15" t="str">
         <x:v>LOR-QUOTATION</x:v>
       </x:c>
@@ -2174,10 +2203,11 @@
     <x:mergeCell ref="A36:H36"/>
     <x:mergeCell ref="B37:E37"/>
     <x:mergeCell ref="B3:E3"/>
-    <x:mergeCell ref="B4:E4"/>
     <x:mergeCell ref="B5:E5"/>
+    <x:mergeCell ref="B4:D4"/>
+    <x:mergeCell ref="E4:F4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fb6cb734d3d4df5"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cca8792a5b74614"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Adjust quotation header font sizes
</commit_message>
<xml_diff>
--- a/public/quotation-template.xlsx
+++ b/public/quotation-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotation" sheetId="1" r:id="R0fd40f4dea194b41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotation" sheetId="1" r:id="Ra3f31c0fdcd54ed6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="181" formatCode="m/d/yy;@"/>
     <x:numFmt numFmtId="182" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </x:numFmts>
-  <x:fonts count="50">
+  <x:fonts count="53">
     <x:font>
       <x:sz val="10"/>
       <x:name val="Arial"/>
@@ -288,6 +288,22 @@
     <x:font>
       <x:sz val="8"/>
       <x:color rgb="FFA6A6A6"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="8.5"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="8.5"/>
+      <x:color rgb="FF111111"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -765,7 +781,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="166">
+  <x:cellXfs count="169">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -1241,6 +1257,15 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="47" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="50" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="49">
@@ -1388,7 +1413,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re34641f6b8fe4e78"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5297f9f9ac3a4a0b"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1420,7 +1445,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R27132b28be62416e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0414350525094a06"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1674,7 +1699,7 @@
       </x:c>
     </x:row>
     <x:row r="3" s="1" customFormat="1" customHeight="1">
-      <x:c r="B3" s="155" t="str">
+      <x:c r="B3" s="166" t="str">
         <x:v>LORIOT INDUSTRIAL CO., LTD</x:v>
       </x:c>
       <x:c r="C3" s="155"/>
@@ -1682,21 +1707,21 @@
       <x:c r="E3" s="155"/>
     </x:row>
     <x:row r="4" s="2" customFormat="1" customHeight="1">
-      <x:c r="B4" s="158" t="str">
+      <x:c r="B4" s="167" t="str">
         <x:v>129 TAN CANG STR, THANH MY TAY WARD, HCMC</x:v>
       </x:c>
       <x:c r="C4" s="158"/>
-      <x:c r="D4" s="155"/>
-      <x:c r="E4" s="164" t="str">
+      <x:c r="D4" s="162" t="str">
         <x:v>QUOTATION NO.</x:v>
       </x:c>
+      <x:c r="E4" s="164"/>
       <x:c r="F4" s="162"/>
       <x:c r="G4" s="15" t="str">
         <x:v>LOR-QUOTATION</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="2" customFormat="1" customHeight="1">
-      <x:c r="B5" s="156" t="str">
+      <x:c r="B5" s="168" t="str">
         <x:v>TEL: +84-28-3899 1163          FAX: +84-28-3899 1189</x:v>
       </x:c>
       <x:c r="C5" s="156"/>
@@ -2204,10 +2229,10 @@
     <x:mergeCell ref="B37:E37"/>
     <x:mergeCell ref="B3:E3"/>
     <x:mergeCell ref="B5:E5"/>
-    <x:mergeCell ref="B4:D4"/>
-    <x:mergeCell ref="E4:F4"/>
+    <x:mergeCell ref="B4:C4"/>
+    <x:mergeCell ref="D4:F4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cca8792a5b74614"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0eebe21f0b34dad"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Use upright quotation address text
</commit_message>
<xml_diff>
--- a/public/quotation-template.xlsx
+++ b/public/quotation-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotation" sheetId="1" r:id="Ra3f31c0fdcd54ed6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotation" sheetId="1" r:id="R0b7a45a9f8674427"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +25,7 @@
     <x:numFmt numFmtId="181" formatCode="m/d/yy;@"/>
     <x:numFmt numFmtId="182" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </x:numFmts>
-  <x:fonts count="53">
+  <x:fonts count="56">
     <x:font>
       <x:sz val="10"/>
       <x:name val="Arial"/>
@@ -297,6 +297,21 @@
     </x:font>
     <x:font>
       <x:i/>
+      <x:sz val="8"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="8"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="8"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
       <x:sz val="8.5"/>
       <x:color rgb="FF111111"/>
       <x:name val="Arial"/>
@@ -781,7 +796,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="169">
+  <x:cellXfs count="172">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -1265,6 +1280,15 @@
       <x:alignment horizontal="left" vertical="center" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="53" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="54" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
@@ -1413,7 +1437,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5297f9f9ac3a4a0b"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8e11c3a19c654750"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1445,7 +1469,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0414350525094a06"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R344f5a49f83f485e"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1707,7 +1731,7 @@
       <x:c r="E3" s="155"/>
     </x:row>
     <x:row r="4" s="2" customFormat="1" customHeight="1">
-      <x:c r="B4" s="167" t="str">
+      <x:c r="B4" s="170" t="str">
         <x:v>129 TAN CANG STR, THANH MY TAY WARD, HCMC</x:v>
       </x:c>
       <x:c r="C4" s="158"/>
@@ -1721,7 +1745,7 @@
       </x:c>
     </x:row>
     <x:row r="5" s="2" customFormat="1" customHeight="1">
-      <x:c r="B5" s="168" t="str">
+      <x:c r="B5" s="171" t="str">
         <x:v>TEL: +84-28-3899 1163          FAX: +84-28-3899 1189</x:v>
       </x:c>
       <x:c r="C5" s="156"/>
@@ -2233,6 +2257,6 @@
     <x:mergeCell ref="D4:F4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0eebe21f0b34dad"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4f2bd075f8f4882"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Format quotation expiration date with month name
</commit_message>
<xml_diff>
--- a/public/quotation-template.xlsx
+++ b/public/quotation-template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotation" sheetId="1" r:id="R0b7a45a9f8674427"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quotation" sheetId="1" r:id="R7f7c4d2eb2c5460d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +13,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="10">
+  <x:numFmts count="11">
     <x:numFmt numFmtId="41" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;_);_(@_)"/>
     <x:numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <x:numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
@@ -24,8 +24,9 @@
     <x:numFmt numFmtId="180" formatCode="[$-409]dd\-mmm\-yy;@"/>
     <x:numFmt numFmtId="181" formatCode="m/d/yy;@"/>
     <x:numFmt numFmtId="182" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <x:numFmt numFmtId="200" formatCode="[$-409]dd\-mmm\-yyyy;@"/>
   </x:numFmts>
-  <x:fonts count="56">
+  <x:fonts count="58">
     <x:font>
       <x:sz val="10"/>
       <x:name val="Arial"/>
@@ -297,6 +298,16 @@
     </x:font>
     <x:font>
       <x:i/>
+      <x:sz val="8"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="8"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
       <x:sz val="8"/>
       <x:color rgb="FF111111"/>
       <x:name val="Arial"/>
@@ -796,7 +807,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="172">
+  <x:cellXfs count="175">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -1289,6 +1300,15 @@
       <x:alignment horizontal="left" vertical="center" wrapText="0"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="56" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="57" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
@@ -1437,7 +1457,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8e11c3a19c654750"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0ca2eff51d2c4e3c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1469,7 +1489,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R344f5a49f83f485e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2856718fddac46fa"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -1731,7 +1751,7 @@
       <x:c r="E3" s="155"/>
     </x:row>
     <x:row r="4" s="2" customFormat="1" customHeight="1">
-      <x:c r="B4" s="170" t="str">
+      <x:c r="B4" s="173" t="str">
         <x:v>129 TAN CANG STR, THANH MY TAY WARD, HCMC</x:v>
       </x:c>
       <x:c r="C4" s="158"/>
@@ -1745,7 +1765,7 @@
       </x:c>
     </x:row>
     <x:row r="5" s="2" customFormat="1" customHeight="1">
-      <x:c r="B5" s="171" t="str">
+      <x:c r="B5" s="174" t="str">
         <x:v>TEL: +84-28-3899 1163          FAX: +84-28-3899 1189</x:v>
       </x:c>
       <x:c r="C5" s="156"/>
@@ -1781,7 +1801,7 @@
           <x:t xml:space="preserve">EXPIRATION DATE</x:t>
         </x:is>
       </x:c>
-      <x:c r="G7" s="19" t="str"/>
+      <x:c r="G7" s="172" t="str"/>
       <x:c r="H7" s="19"/>
     </x:row>
     <x:row r="8" s="2" customFormat="1" customHeight="1">
@@ -2257,6 +2277,6 @@
     <x:mergeCell ref="D4:F4"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4f2bd075f8f4882"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbc5ee8f5f6f243b5"/>
 </x:worksheet>
 </file>
</xml_diff>